<commit_message>
feat: CharacterTID 1 폐기 (영구 결번)
- CharacterTable에서 TID 1 '기본 캐릭터' 행 삭제, 이제 1001~1006 6행
- 기존 계정은 다음 로그인에 1001을 자동 지급받는다
  (LoadCharacters가 없는 TID를 건너뛰어 0명이 되고, 그때 지급 경로가 돈다)
- 캐릭터 기획안 3.3 · 게임기획코어 확정 현황을 실행 완료로 갱신
</commit_message>
<xml_diff>
--- a/GameDesign/Excel/Character.xlsx
+++ b/GameDesign/Excel/Character.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:I16"/>
+  <dimension ref="A2:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="2"/>
@@ -808,11 +808,11 @@
     </row>
     <row r="10">
       <c r="B10" t="n">
-        <v>1</v>
+        <v>1001</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>기본 캐릭터</t>
+          <t>램볼</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -832,185 +832,155 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>기본 지급. 2~1000번은 예약 대역, 일반 캐릭터는 1001부터</t>
+          <t>시작 지급. 전 산업 1 — 어떤 산업이든 시작할 수 있어야 한다</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="n">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>램볼</t>
+          <t>치키피</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>시작 지급. 전 산업 1 — 어떤 산업이든 시작할 수 있어야 한다</t>
+          <t>농사 담당</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="n">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>치키피</t>
+          <t>펭구렛</t>
         </is>
       </c>
       <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
         <v>3</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
       <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
         <v>2</v>
       </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>농사 담당</t>
+          <t>낚시 담당</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="n">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>펭구렛</t>
+          <t>캐티바</t>
         </is>
       </c>
       <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" t="n">
         <v>1</v>
       </c>
-      <c r="E13" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
       <c r="H13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>낚시 담당</t>
+          <t>채굴 담당</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="n">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>캐티바</t>
+          <t>리프몽</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
         <v>0</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>3</v>
       </c>
-      <c r="G14" t="n">
-        <v>1</v>
-      </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>채굴 담당</t>
+          <t>벌목 담당</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="n">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>리프몽</t>
+          <t>폭스파크스</t>
         </is>
       </c>
       <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="n">
         <v>1</v>
       </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>0</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>3</v>
       </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
       <c r="I15" t="inlineStr">
-        <is>
-          <t>벌목 담당</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" t="n">
-        <v>1006</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>폭스파크스</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>2</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>3</v>
-      </c>
-      <c r="I16" t="inlineStr">
         <is>
           <t>사냥 담당</t>
         </is>

</xml_diff>